<commit_message>
Rewrite bug titles in what-where-when passive form
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-test-cases/Demo_bug_reports.xlsx
+++ b/demo-test-cases/Demo_bug_reports.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>problem_user: all product images are missing in the catalog</t>
+          <t>Product images are not displayed on the Products page after login as problem_user</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>problem_user: sorting does not work</t>
+          <t>Products are not sorted on the Products page when a sort option is selected by problem_user</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Add to cart does not work for 3 of 6 products (problem_user and error_user)</t>
+          <t>Products are not added to the cart when "Add to cart" is clicked for 3 of 6 products (problem_user, error_user)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>problem_user: typing the last name overwrites the first name on checkout</t>
+          <t>First Name is overwritten on the Checkout page when Last Name is entered by problem_user</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>error_user: Last Name field does not accept input and checkout skips its validation</t>
+          <t>Last Name input is not accepted and its validation is skipped on the Checkout page when Continue is clicked by error_user</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>error_user: Finish button does not complete the order</t>
+          <t>Order is not completed on the Checkout Overview page when Finish is clicked by error_user</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove Environment column from bug reports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-test-cases/Demo_bug_reports.xlsx
+++ b/demo-test-cases/Demo_bug_reports.xlsx
@@ -450,18 +450,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,35 +476,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Preconditions</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Preconditions</t>
+          <t>Steps to reproduce</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Steps to reproduce</t>
+          <t>Actual result</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Actual result</t>
+          <t>Expected result</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Expected result</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Attachment</t>
         </is>
@@ -524,36 +518,31 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>https://www.saucedemo.com, Chromium (desktop, 1280x900), Windows 11, checked on 24 Oct 2026</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Login page is open</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>1. Log in as problem_user / secret_sauce
 2. Look at the Products page</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>All 6 products use the same placeholder file (sl-404.jpg). Images are not displayed, only empty space is shown next to each product.</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>All 6 products use the same placeholder file (sl-404.jpg). Images are not displayed, only empty space is shown next to each product.</t>
+          <t>Each product shows its own image.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Each product shows its own image.</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>bug-evidence/problem_user_catalog_images.png</t>
         </is>
@@ -572,35 +561,30 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://www.saucedemo.com, Chromium (desktop, 1280x900), Windows 11, checked on 24 Oct 2026</t>
+          <t>User is logged in as problem_user, Products page is open</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>User is logged in as problem_user, Products page is open</t>
+          <t>1. Select "Name (Z to A)" in the sort dropdown</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1. Select "Name (Z to A)" in the sort dropdown</t>
+          <t>Product order does not change (stays A to Z). The dropdown returns to "Name (A to Z)".</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Product order does not change (stays A to Z). The dropdown returns to "Name (A to Z)".</t>
+          <t>Products are sorted from Z to A and the dropdown keeps the selected option.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Products are sorted from Z to A and the dropdown keeps the selected option.</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>bug-evidence/problem_user_sort_za.png</t>
         </is>
@@ -619,37 +603,32 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://www.saucedemo.com, Chromium (desktop, 1280x900), Windows 11, checked on 24 Oct 2026</t>
+          <t>User is logged in as problem_user (same result for error_user), cart is empty</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in as problem_user (same result for error_user), cart is empty</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>1. Click "Add to cart" on Sauce Labs Bolt T-Shirt
 2. Click "Add to cart" on Sauce Labs Fleece Jacket
 3. Click "Add to cart" on Test.allTheThings() T-Shirt (Red)</t>
         </is>
       </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>The button stays "Add to cart" and the cart badge does not increase for these 3 products. The other 3 products (Backpack, Bike Light, Onesie) are added correctly.</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>The button stays "Add to cart" and the cart badge does not increase for these 3 products. The other 3 products (Backpack, Bike Light, Onesie) are added correctly.</t>
+          <t>Each click adds the product, the button changes to "Remove" and the badge increases by 1.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Each click adds the product, the button changes to "Remove" and the badge increases by 1.</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>bug-evidence/problem_user_add_to_cart.png, bug-evidence/error_user_add_to_cart.png</t>
         </is>
@@ -668,15 +647,10 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://www.saucedemo.com, Chromium (desktop, 1280x900), Windows 11, checked on 24 Oct 2026</t>
+          <t>User is logged in as problem_user, cart has a product, checkout step one page is open</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in as problem_user, cart has a product, checkout step one page is open</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>1. Enter "Test" in First Name
 2. Enter "User" in Last Name
@@ -684,22 +658,22 @@
 4. Click Continue</t>
         </is>
       </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>First Name field shows "User" and Last Name stays empty. Error "Last Name is required" is shown, so the order cannot continue.</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>First Name field shows "User" and Last Name stays empty. Error "Last Name is required" is shown, so the order cannot continue.</t>
+          <t>Each field keeps the value typed into it and the user proceeds to the overview page.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Each field keeps the value typed into it and the user proceeds to the overview page.</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>bug-evidence/problem_user_checkout_form.png</t>
         </is>
@@ -718,15 +692,10 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.saucedemo.com, Chromium (desktop, 1280x900), Windows 11, checked on 24 Oct 2026</t>
+          <t>User is logged in as error_user, cart has a product, checkout step one page is open</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in as error_user, cart has a product, checkout step one page is open</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>1. Enter "Test" in First Name
 2. Enter "User" in Last Name
@@ -734,22 +703,22 @@
 4. Click Continue</t>
         </is>
       </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Last Name stays empty after typing. No error is shown and the user is taken to the overview page with an empty last name.</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Last Name stays empty after typing. No error is shown and the user is taken to the overview page with an empty last name.</t>
+          <t>Last Name keeps the typed value. If it is empty, error "Last Name is required" is shown.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Last Name keeps the typed value. If it is empty, error "Last Name is required" is shown.</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>bug-evidence/error_user_checkout_form.png</t>
         </is>
@@ -768,35 +737,30 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>https://www.saucedemo.com, Chromium (desktop, 1280x900), Windows 11, checked on 24 Oct 2026</t>
+          <t>User is logged in as error_user, checkout overview page is open (reached with the steps from BUG-05)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>User is logged in as error_user, checkout overview page is open (reached with the steps from BUG-05)</t>
+          <t>1. Click Finish</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1. Click Finish</t>
+          <t>Nothing happens. The user stays on the overview page, no confirmation "Thank you for your order" is shown and the cart badge still shows 1.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Nothing happens. The user stays on the overview page, no confirmation "Thank you for your order" is shown and the cart badge still shows 1.</t>
+          <t>The order is completed and the confirmation page is shown.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>The order is completed and the confirmation page is shown.</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>bug-evidence/error_user_finish.png</t>
         </is>

</xml_diff>

<commit_message>
Remove Severity and Attachment columns from bug reports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-test-cases/Demo_bug_reports.xlsx
+++ b/demo-test-cases/Demo_bug_reports.xlsx
@@ -450,17 +450,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,16 +492,6 @@
           <t>Expected result</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Attachment</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -537,16 +525,6 @@
           <t>Each product shows its own image.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>bug-evidence/problem_user_catalog_images.png</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -577,16 +555,6 @@
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Products are sorted from Z to A and the dropdown keeps the selected option.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>bug-evidence/problem_user_sort_za.png</t>
         </is>
       </c>
     </row>
@@ -621,16 +589,6 @@
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Each click adds the product, the button changes to "Remove" and the badge increases by 1.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>bug-evidence/problem_user_add_to_cart.png, bug-evidence/error_user_add_to_cart.png</t>
         </is>
       </c>
     </row>
@@ -668,16 +626,6 @@
           <t>Each field keeps the value typed into it and the user proceeds to the overview page.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>bug-evidence/problem_user_checkout_form.png</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -713,16 +661,6 @@
           <t>Last Name keeps the typed value. If it is empty, error "Last Name is required" is shown.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>bug-evidence/error_user_checkout_form.png</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -753,16 +691,6 @@
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>The order is completed and the confirmation page is shown.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>bug-evidence/error_user_finish.png</t>
         </is>
       </c>
     </row>
@@ -811,7 +739,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>The site has special demo users (problem_user, error_user) with intentionally seeded defects. All reports above were reproduced by running the steps, screenshots are in the bug-evidence folder.</t>
+          <t>The site has special demo users (problem_user, error_user) with intentionally seeded defects. All reports above were reproduced by running the steps.</t>
         </is>
       </c>
     </row>
@@ -823,7 +751,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>To show how I describe defects: exact steps, actual and expected result, severity and evidence.</t>
+          <t>To show how I describe defects: clear title, exact steps, actual and expected result.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove About sheet from bug reports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-test-cases/Demo_bug_reports.xlsx
+++ b/demo-test-cases/Demo_bug_reports.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug reports" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -73,16 +72,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -697,65 +692,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Sample bug reports</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Application</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>https://www.saucedemo.com (public demo shop made for testing practice)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Source of defects</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>The site has special demo users (problem_user, error_user) with intentionally seeded defects. All reports above were reproduced by running the steps.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>To show how I describe defects: clear title, exact steps, actual and expected result.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Use generic 'user' in bug titles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-test-cases/Demo_bug_reports.xlsx
+++ b/demo-test-cases/Demo_bug_reports.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product images are not displayed on the Products page after login as problem_user</t>
+          <t>Product images are not displayed on the Products page after login by user</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Products are not sorted on the Products page when a sort option is selected by problem_user</t>
+          <t>Products are not sorted on the Products page when a sort option is selected by user</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Products are not added to the cart when "Add to cart" is clicked for 3 of 6 products (problem_user, error_user)</t>
+          <t>Products are not added to the cart when "Add to cart" is clicked for 3 of 6 products by user</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>First Name is overwritten on the Checkout page when Last Name is entered by problem_user</t>
+          <t>First Name is overwritten on the Checkout page when Last Name is entered by user</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Last Name input is not accepted and its validation is skipped on the Checkout page when Continue is clicked by error_user</t>
+          <t>Last Name input is not accepted and its validation is skipped on the Checkout page when Continue is clicked by user</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Order is not completed on the Checkout Overview page when Finish is clicked by error_user</t>
+          <t>Order is not completed on the Checkout Overview page when Finish is clicked by user</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">

</xml_diff>